<commit_message>
v13.66: docs(cupia): 과제2 견적서 20260731 — NSHC 표준 양식 기반 (EWACS AI Agent 22 M/M, 역할 5종 직무별 단가, 합계 193,481,808원 VAT별도, 과제1은 수행 완료로 제외, 발행주체 (주)씨커스/Seekers Inc. 표기) + 견적 양식·AI 공동연구방안 PDF reference 등재(05·06) + 관리대장 CT-03 갱신
</commit_message>
<xml_diff>
--- a/cupia-ai-research/docs/00_산출물관리/산출물_관리대장_v0.1.xlsx
+++ b/cupia-ai-research/docs/00_산출물관리/산출물_관리대장_v0.1.xlsx
@@ -692,12 +692,12 @@
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>예정</t>
+          <t>초안 20260731 (과제2 한정)</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>CUPIA 예산 확인 후 — M/M 단가표 포함</t>
+          <t>08_계약관리/ — 22 M/M·193,481,808원(VAT별도), 양식: reference/05, 과제1은 수행 완료로 제외</t>
         </is>
       </c>
     </row>

</xml_diff>